<commit_message>
Combined scan results 2026-10-14
</commit_message>
<xml_diff>
--- a/results/2026-10-14.xlsx
+++ b/results/2026-10-14.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E49"/>
+  <dimension ref="A1:E50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -452,37 +452,41 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>AEP</t>
+          <t>AR</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>AFRM</t>
+          <t>AAPL</t>
         </is>
       </c>
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>AAPL</t>
+          <t>AFRM</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr"/>
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>PNFP</t>
+        </is>
+      </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>ANIP</t>
+          <t>CINF</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>AMGN</t>
+          <t>ADP</t>
         </is>
       </c>
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>ARQT</t>
+          <t>AVPT</t>
         </is>
       </c>
     </row>
@@ -490,12 +494,12 @@
       <c r="A4" t="inlineStr"/>
       <c r="B4" t="inlineStr">
         <is>
-          <t>AR</t>
+          <t>COCO</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>AMZN</t>
+          <t>ALLT</t>
         </is>
       </c>
       <c r="D4" t="inlineStr"/>
@@ -509,18 +513,18 @@
       <c r="A5" t="inlineStr"/>
       <c r="B5" t="inlineStr">
         <is>
-          <t>CINF</t>
+          <t>ENSG</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>APA</t>
+          <t>AMGN</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>BTSG</t>
+          <t>DAVE</t>
         </is>
       </c>
     </row>
@@ -528,18 +532,18 @@
       <c r="A6" t="inlineStr"/>
       <c r="B6" t="inlineStr">
         <is>
-          <t>COCO</t>
+          <t>ERIC</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>AVPT</t>
+          <t>AMZN</t>
         </is>
       </c>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>CDNS</t>
+          <t>DLO</t>
         </is>
       </c>
     </row>
@@ -547,18 +551,18 @@
       <c r="A7" t="inlineStr"/>
       <c r="B7" t="inlineStr">
         <is>
-          <t>ENSG</t>
+          <t>EXC</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>BIIB</t>
+          <t>APA</t>
         </is>
       </c>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>CGNX</t>
+          <t>EXEL</t>
         </is>
       </c>
     </row>
@@ -566,18 +570,18 @@
       <c r="A8" t="inlineStr"/>
       <c r="B8" t="inlineStr">
         <is>
-          <t>ERIC</t>
+          <t>EXE</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>CAKE</t>
+          <t>ARQT</t>
         </is>
       </c>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>CORT</t>
+          <t>LOGI</t>
         </is>
       </c>
     </row>
@@ -585,18 +589,18 @@
       <c r="A9" t="inlineStr"/>
       <c r="B9" t="inlineStr">
         <is>
-          <t>EXC</t>
+          <t>FELE</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>CLOV</t>
+          <t>BIIB</t>
         </is>
       </c>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>CSCO</t>
+          <t>NTAP</t>
         </is>
       </c>
     </row>
@@ -604,18 +608,18 @@
       <c r="A10" t="inlineStr"/>
       <c r="B10" t="inlineStr">
         <is>
-          <t>EXE</t>
+          <t>FUTU</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>CME</t>
+          <t>CAKE</t>
         </is>
       </c>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>DDOG</t>
+          <t>OKTA</t>
         </is>
       </c>
     </row>
@@ -623,18 +627,18 @@
       <c r="A11" t="inlineStr"/>
       <c r="B11" t="inlineStr">
         <is>
-          <t>FELE</t>
+          <t>HTHT</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>COKE</t>
+          <t>CART</t>
         </is>
       </c>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>EXTR</t>
+          <t>PCVX</t>
         </is>
       </c>
     </row>
@@ -642,18 +646,18 @@
       <c r="A12" t="inlineStr"/>
       <c r="B12" t="inlineStr">
         <is>
-          <t>FUTU</t>
+          <t>IDXX</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>COR</t>
+          <t>CLMT</t>
         </is>
       </c>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
-          <t>FFIV</t>
+          <t>QLYS</t>
         </is>
       </c>
     </row>
@@ -661,18 +665,18 @@
       <c r="A13" t="inlineStr"/>
       <c r="B13" t="inlineStr">
         <is>
-          <t>GPGI</t>
+          <t>LNT</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>CR</t>
+          <t>CLOV</t>
         </is>
       </c>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
-          <t>FLEX</t>
+          <t>RELY</t>
         </is>
       </c>
     </row>
@@ -680,18 +684,18 @@
       <c r="A14" t="inlineStr"/>
       <c r="B14" t="inlineStr">
         <is>
-          <t>HON</t>
+          <t>NXT</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>CTAS</t>
+          <t>CME</t>
         </is>
       </c>
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
-          <t>FTNT</t>
+          <t>RZLT</t>
         </is>
       </c>
     </row>
@@ -699,18 +703,18 @@
       <c r="A15" t="inlineStr"/>
       <c r="B15" t="inlineStr">
         <is>
-          <t>HTHT</t>
+          <t>ODFL</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>CVLT</t>
+          <t>COKE</t>
         </is>
       </c>
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
-          <t>GILD</t>
+          <t>SYNA</t>
         </is>
       </c>
     </row>
@@ -718,18 +722,18 @@
       <c r="A16" t="inlineStr"/>
       <c r="B16" t="inlineStr">
         <is>
-          <t>IDXX</t>
+          <t>ORLY</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>DAVE</t>
+          <t>COR</t>
         </is>
       </c>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
-          <t>IBRX</t>
+          <t>UTHR</t>
         </is>
       </c>
     </row>
@@ -737,265 +741,193 @@
       <c r="A17" t="inlineStr"/>
       <c r="B17" t="inlineStr">
         <is>
-          <t>LNT</t>
+          <t>PECO</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>DLO</t>
+          <t>CTAS</t>
         </is>
       </c>
       <c r="D17" t="inlineStr"/>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>IDCC</t>
-        </is>
-      </c>
+      <c r="E17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr"/>
       <c r="B18" t="inlineStr">
         <is>
-          <t>LSTR</t>
+          <t>REAL</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>EBAY</t>
+          <t>CVLT</t>
         </is>
       </c>
       <c r="D18" t="inlineStr"/>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>IOVA</t>
-        </is>
-      </c>
+      <c r="E18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr"/>
       <c r="B19" t="inlineStr">
         <is>
-          <t>NXT</t>
+          <t>REG</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>EXEL</t>
+          <t>DBX</t>
         </is>
       </c>
       <c r="D19" t="inlineStr"/>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>KOD</t>
-        </is>
-      </c>
+      <c r="E19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr"/>
       <c r="B20" t="inlineStr">
         <is>
-          <t>ODFL</t>
+          <t>SUPN</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>FAST</t>
+          <t>EBAY</t>
         </is>
       </c>
       <c r="D20" t="inlineStr"/>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>LGND</t>
-        </is>
-      </c>
+      <c r="E20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr"/>
       <c r="B21" t="inlineStr">
         <is>
-          <t>ORLY</t>
+          <t>VMRK</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>GCT</t>
+          <t>EVRG</t>
         </is>
       </c>
       <c r="D21" t="inlineStr"/>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>MEDP</t>
-        </is>
-      </c>
+      <c r="E21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr"/>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>PECO</t>
-        </is>
-      </c>
+      <c r="B22" t="inlineStr"/>
       <c r="C22" t="inlineStr">
         <is>
-          <t>GMAB</t>
+          <t>FAST</t>
         </is>
       </c>
       <c r="D22" t="inlineStr"/>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>MEOH</t>
-        </is>
-      </c>
+      <c r="E22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr"/>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>PNFP</t>
-        </is>
-      </c>
+      <c r="B23" t="inlineStr"/>
       <c r="C23" t="inlineStr">
         <is>
-          <t>GOOG</t>
+          <t>FROG</t>
         </is>
       </c>
       <c r="D23" t="inlineStr"/>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>NTAP</t>
-        </is>
-      </c>
+      <c r="E23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr"/>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>REG</t>
-        </is>
-      </c>
+      <c r="B24" t="inlineStr"/>
       <c r="C24" t="inlineStr">
         <is>
-          <t>GOOGL</t>
+          <t>GOOG</t>
         </is>
       </c>
       <c r="D24" t="inlineStr"/>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>NTNX</t>
-        </is>
-      </c>
+      <c r="E24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr"/>
       <c r="B25" t="inlineStr"/>
       <c r="C25" t="inlineStr">
         <is>
-          <t>HAS</t>
+          <t>GOOGL</t>
         </is>
       </c>
       <c r="D25" t="inlineStr"/>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>NWE</t>
-        </is>
-      </c>
+      <c r="E25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr"/>
       <c r="B26" t="inlineStr"/>
       <c r="C26" t="inlineStr">
         <is>
-          <t>HURN</t>
+          <t>HAS</t>
         </is>
       </c>
       <c r="D26" t="inlineStr"/>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
+      <c r="E26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr"/>
       <c r="B27" t="inlineStr"/>
       <c r="C27" t="inlineStr">
         <is>
-          <t>JOYY</t>
+          <t>HURN</t>
         </is>
       </c>
       <c r="D27" t="inlineStr"/>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>PCVX</t>
-        </is>
-      </c>
+      <c r="E27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr"/>
       <c r="B28" t="inlineStr"/>
       <c r="C28" t="inlineStr">
         <is>
-          <t>KDP</t>
+          <t>JOYY</t>
         </is>
       </c>
       <c r="D28" t="inlineStr"/>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t>STLN</t>
-        </is>
-      </c>
+      <c r="E28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr"/>
       <c r="B29" t="inlineStr"/>
       <c r="C29" t="inlineStr">
         <is>
-          <t>KNSA</t>
+          <t>KDP</t>
         </is>
       </c>
       <c r="D29" t="inlineStr"/>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>SYNA</t>
-        </is>
-      </c>
+      <c r="E29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr"/>
       <c r="B30" t="inlineStr"/>
       <c r="C30" t="inlineStr">
         <is>
-          <t>LAUR</t>
+          <t>KNSA</t>
         </is>
       </c>
       <c r="D30" t="inlineStr"/>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>UTHR</t>
-        </is>
-      </c>
+      <c r="E30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr"/>
       <c r="B31" t="inlineStr"/>
       <c r="C31" t="inlineStr">
         <is>
-          <t>MAR</t>
+          <t>LAUR</t>
         </is>
       </c>
       <c r="D31" t="inlineStr"/>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t>XNCR</t>
-        </is>
-      </c>
+      <c r="E31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr"/>
       <c r="B32" t="inlineStr"/>
       <c r="C32" t="inlineStr">
         <is>
-          <t>MRNA</t>
+          <t>LFST</t>
         </is>
       </c>
       <c r="D32" t="inlineStr"/>
@@ -1006,7 +938,7 @@
       <c r="B33" t="inlineStr"/>
       <c r="C33" t="inlineStr">
         <is>
-          <t>MSFT</t>
+          <t>LGND</t>
         </is>
       </c>
       <c r="D33" t="inlineStr"/>
@@ -1017,7 +949,7 @@
       <c r="B34" t="inlineStr"/>
       <c r="C34" t="inlineStr">
         <is>
-          <t>MTCH</t>
+          <t>MAR</t>
         </is>
       </c>
       <c r="D34" t="inlineStr"/>
@@ -1028,7 +960,7 @@
       <c r="B35" t="inlineStr"/>
       <c r="C35" t="inlineStr">
         <is>
-          <t>NDSN</t>
+          <t>MEOH</t>
         </is>
       </c>
       <c r="D35" t="inlineStr"/>
@@ -1039,7 +971,7 @@
       <c r="B36" t="inlineStr"/>
       <c r="C36" t="inlineStr">
         <is>
-          <t>OKTA</t>
+          <t>MSFT</t>
         </is>
       </c>
       <c r="D36" t="inlineStr"/>
@@ -1050,7 +982,7 @@
       <c r="B37" t="inlineStr"/>
       <c r="C37" t="inlineStr">
         <is>
-          <t>OPLN</t>
+          <t>MTCH</t>
         </is>
       </c>
       <c r="D37" t="inlineStr"/>
@@ -1061,7 +993,7 @@
       <c r="B38" t="inlineStr"/>
       <c r="C38" t="inlineStr">
         <is>
-          <t>PENG</t>
+          <t>NWE</t>
         </is>
       </c>
       <c r="D38" t="inlineStr"/>
@@ -1072,7 +1004,7 @@
       <c r="B39" t="inlineStr"/>
       <c r="C39" t="inlineStr">
         <is>
-          <t>PLTR</t>
+          <t>OPLN</t>
         </is>
       </c>
       <c r="D39" t="inlineStr"/>
@@ -1083,7 +1015,7 @@
       <c r="B40" t="inlineStr"/>
       <c r="C40" t="inlineStr">
         <is>
-          <t>PRCH</t>
+          <t>PENG</t>
         </is>
       </c>
       <c r="D40" t="inlineStr"/>
@@ -1094,7 +1026,7 @@
       <c r="B41" t="inlineStr"/>
       <c r="C41" t="inlineStr">
         <is>
-          <t>RELL</t>
+          <t>PLTR</t>
         </is>
       </c>
       <c r="D41" t="inlineStr"/>
@@ -1105,7 +1037,7 @@
       <c r="B42" t="inlineStr"/>
       <c r="C42" t="inlineStr">
         <is>
-          <t>RZLT</t>
+          <t>PRCH</t>
         </is>
       </c>
       <c r="D42" t="inlineStr"/>
@@ -1127,7 +1059,7 @@
       <c r="B44" t="inlineStr"/>
       <c r="C44" t="inlineStr">
         <is>
-          <t>SHOP</t>
+          <t>SEZL</t>
         </is>
       </c>
       <c r="D44" t="inlineStr"/>
@@ -1138,7 +1070,7 @@
       <c r="B45" t="inlineStr"/>
       <c r="C45" t="inlineStr">
         <is>
-          <t>SKWD</t>
+          <t>SHOP</t>
         </is>
       </c>
       <c r="D45" t="inlineStr"/>
@@ -1171,7 +1103,7 @@
       <c r="B48" t="inlineStr"/>
       <c r="C48" t="inlineStr">
         <is>
-          <t>TRMD</t>
+          <t>STLN</t>
         </is>
       </c>
       <c r="D48" t="inlineStr"/>
@@ -1182,11 +1114,22 @@
       <c r="B49" t="inlineStr"/>
       <c r="C49" t="inlineStr">
         <is>
-          <t>VSXY</t>
+          <t>TRMD</t>
         </is>
       </c>
       <c r="D49" t="inlineStr"/>
       <c r="E49" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr"/>
+      <c r="B50" t="inlineStr"/>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>VSXY</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr"/>
+      <c r="E50" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1199,7 +1142,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:D9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1227,12 +1170,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>FAST</t>
+          <t>APA</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>ECHO</t>
+          <t>AAPL</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -1242,137 +1185,111 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>APA</t>
+          <t>GOOGL</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>OPCH</t>
+          <t>GILD</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>CRWD</t>
+          <t>BORR</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>MSFT</t>
+          <t>GTLB</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>GOOGL</t>
+          <t>PLTR</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>PENG</t>
+          <t>IBRX</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>EBAY</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>PANW</t>
-        </is>
-      </c>
+          <t>SHOP</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr">
         <is>
-          <t>GTLB</t>
+          <t>SUNB</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>SHOP</t>
+          <t>LYFT</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>EXEL</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>TRMD</t>
-        </is>
-      </c>
+          <t>OPCH</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr">
         <is>
-          <t>MAT</t>
+          <t>MRNA</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>SPCX</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>GMAB</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>VYLR</t>
-        </is>
-      </c>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr"/>
+      <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr">
         <is>
-          <t>PTC</t>
+          <t>P</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>FRSH</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>SUNB</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>OKTA</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>NTSK</t>
-        </is>
-      </c>
+          <t>PYPL</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr"/>
+      <c r="C7" t="inlineStr"/>
+      <c r="D7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>PLTR</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>TECH</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>AFRM</t>
-        </is>
-      </c>
+          <t>PENG</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr"/>
+      <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>INTR</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr"/>
+      <c r="C9" t="inlineStr"/>
+      <c r="D9" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>